<commit_message>
working OR tools with barely working flowchart
</commit_message>
<xml_diff>
--- a/Server/uploaded_data.xlsx
+++ b/Server/uploaded_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="71">
   <si>
     <t>employee_id</t>
   </si>
@@ -61,30 +61,30 @@
     <t>E03</t>
   </si>
   <si>
+    <t>any</t>
+  </si>
+  <si>
+    <t>double</t>
+  </si>
+  <si>
     <t>E04</t>
   </si>
   <si>
+    <t>normal</t>
+  </si>
+  <si>
+    <t>triple</t>
+  </si>
+  <si>
     <t>E05</t>
   </si>
   <si>
-    <t>any</t>
-  </si>
-  <si>
-    <t>double</t>
-  </si>
-  <si>
     <t>E06</t>
   </si>
   <si>
     <t>E07</t>
   </si>
   <si>
-    <t>normal</t>
-  </si>
-  <si>
-    <t>triple</t>
-  </si>
-  <si>
     <t>E08</t>
   </si>
   <si>
@@ -94,6 +94,21 @@
     <t>E10</t>
   </si>
   <si>
+    <t>E11</t>
+  </si>
+  <si>
+    <t>E12</t>
+  </si>
+  <si>
+    <t>E13</t>
+  </si>
+  <si>
+    <t>E14</t>
+  </si>
+  <si>
+    <t>E15</t>
+  </si>
+  <si>
     <t>vehicle_id</t>
   </si>
   <si>
@@ -151,6 +166,15 @@
     <t>van</t>
   </si>
   <si>
+    <t>V05</t>
+  </si>
+  <si>
+    <t>2W</t>
+  </si>
+  <si>
+    <t>V06</t>
+  </si>
+  <si>
     <t>baseline_cost</t>
   </si>
   <si>
@@ -166,7 +190,7 @@
     <t>test_case_id</t>
   </si>
   <si>
-    <t>TC_04</t>
+    <t>TC_03</t>
   </si>
   <si>
     <t>city</t>
@@ -203,9 +227,6 @@
   </si>
   <si>
     <t>objective_time_weight</t>
-  </si>
-  <si>
-    <t>infeasible_handling_required</t>
   </si>
 </sst>
 </file>
@@ -530,10 +551,10 @@
         <v>1.0</v>
       </c>
       <c r="C2" s="2">
-        <v>12.936</v>
+        <v>12.9365</v>
       </c>
       <c r="D2" s="2">
-        <v>77.624</v>
+        <v>77.6248</v>
       </c>
       <c r="E2" s="2">
         <v>12.9716</v>
@@ -545,7 +566,7 @@
         <v>0.3402777777777778</v>
       </c>
       <c r="H2" s="3">
-        <v>0.3645833333333333</v>
+        <v>0.375</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>11</v>
@@ -562,10 +583,10 @@
         <v>1.0</v>
       </c>
       <c r="C3" s="2">
-        <v>12.938</v>
+        <v>12.934</v>
       </c>
       <c r="D3" s="2">
-        <v>77.626</v>
+        <v>77.622</v>
       </c>
       <c r="E3" s="2">
         <v>12.9716</v>
@@ -577,7 +598,7 @@
         <v>0.34375</v>
       </c>
       <c r="H3" s="3">
-        <v>0.3680555555555556</v>
+        <v>0.3819444444444444</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>11</v>
@@ -591,13 +612,13 @@
         <v>14</v>
       </c>
       <c r="B4" s="2">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="C4" s="2">
-        <v>12.94</v>
+        <v>12.931</v>
       </c>
       <c r="D4" s="2">
-        <v>77.628</v>
+        <v>77.62</v>
       </c>
       <c r="E4" s="2">
         <v>12.9716</v>
@@ -609,24 +630,24 @@
         <v>0.3472222222222222</v>
       </c>
       <c r="H4" s="3">
-        <v>0.3715277777777778</v>
+        <v>0.3958333333333333</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B5" s="2">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="C5" s="2">
-        <v>12.942</v>
+        <v>12.94</v>
       </c>
       <c r="D5" s="2">
         <v>77.63</v>
@@ -638,30 +659,30 @@
         <v>77.5946</v>
       </c>
       <c r="G5" s="3">
-        <v>0.3506944444444444</v>
+        <v>0.3645833333333333</v>
       </c>
       <c r="H5" s="3">
-        <v>0.375</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B6" s="2">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="C6" s="2">
-        <v>12.93</v>
+        <v>12.918</v>
       </c>
       <c r="D6" s="2">
-        <v>77.62</v>
+        <v>77.61</v>
       </c>
       <c r="E6" s="2">
         <v>12.9716</v>
@@ -670,30 +691,30 @@
         <v>77.5946</v>
       </c>
       <c r="G6" s="3">
-        <v>0.3541666666666667</v>
+        <v>0.3854166666666667</v>
       </c>
       <c r="H6" s="3">
-        <v>0.3958333333333333</v>
+        <v>0.4479166666666667</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B7" s="2">
         <v>2.0</v>
       </c>
       <c r="C7" s="2">
-        <v>12.928</v>
+        <v>12.95</v>
       </c>
       <c r="D7" s="2">
-        <v>77.618</v>
+        <v>77.635</v>
       </c>
       <c r="E7" s="2">
         <v>12.9716</v>
@@ -705,27 +726,27 @@
         <v>0.3541666666666667</v>
       </c>
       <c r="H7" s="3">
-        <v>0.3958333333333333</v>
+        <v>0.40625</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B8" s="2">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="C8" s="2">
-        <v>12.95</v>
+        <v>12.9525</v>
       </c>
       <c r="D8" s="2">
-        <v>77.635</v>
+        <v>77.628</v>
       </c>
       <c r="E8" s="2">
         <v>12.9716</v>
@@ -734,16 +755,16 @@
         <v>77.5946</v>
       </c>
       <c r="G8" s="3">
-        <v>0.3645833333333333</v>
+        <v>0.3368055555555556</v>
       </c>
       <c r="H8" s="3">
-        <v>0.4166666666666667</v>
+        <v>0.375</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -754,10 +775,10 @@
         <v>3.0</v>
       </c>
       <c r="C9" s="2">
-        <v>12.948</v>
+        <v>12.927</v>
       </c>
       <c r="D9" s="2">
-        <v>77.633</v>
+        <v>77.642</v>
       </c>
       <c r="E9" s="2">
         <v>12.9716</v>
@@ -766,16 +787,16 @@
         <v>77.5946</v>
       </c>
       <c r="G9" s="3">
-        <v>0.3645833333333333</v>
+        <v>0.375</v>
       </c>
       <c r="H9" s="3">
-        <v>0.4166666666666667</v>
+        <v>0.4375</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -783,13 +804,13 @@
         <v>24</v>
       </c>
       <c r="B10" s="2">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="C10" s="2">
-        <v>12.915</v>
+        <v>12.941</v>
       </c>
       <c r="D10" s="2">
-        <v>77.605</v>
+        <v>77.631</v>
       </c>
       <c r="E10" s="2">
         <v>12.9716</v>
@@ -798,16 +819,16 @@
         <v>77.5946</v>
       </c>
       <c r="G10" s="3">
-        <v>0.3958333333333333</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="H10" s="3">
-        <v>0.4583333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
@@ -815,13 +836,13 @@
         <v>25</v>
       </c>
       <c r="B11" s="2">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="C11" s="2">
-        <v>13.05</v>
+        <v>12.925</v>
       </c>
       <c r="D11" s="2">
-        <v>77.8</v>
+        <v>77.6</v>
       </c>
       <c r="E11" s="2">
         <v>12.9716</v>
@@ -830,37 +851,177 @@
         <v>77.5946</v>
       </c>
       <c r="G11" s="3">
+        <v>0.3958333333333333</v>
+      </c>
+      <c r="H11" s="3">
+        <v>0.4583333333333333</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="C12" s="2">
+        <v>12.96</v>
+      </c>
+      <c r="D12" s="2">
+        <v>77.64</v>
+      </c>
+      <c r="E12" s="2">
+        <v>12.9716</v>
+      </c>
+      <c r="F12" s="2">
+        <v>77.5946</v>
+      </c>
+      <c r="G12" s="3">
+        <v>0.3611111111111111</v>
+      </c>
+      <c r="H12" s="3">
+        <v>0.4097222222222222</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="C13" s="2">
+        <v>12.933</v>
+      </c>
+      <c r="D13" s="2">
+        <v>77.605</v>
+      </c>
+      <c r="E13" s="2">
+        <v>12.9716</v>
+      </c>
+      <c r="F13" s="2">
+        <v>77.5946</v>
+      </c>
+      <c r="G13" s="3">
+        <v>0.375</v>
+      </c>
+      <c r="H13" s="3">
+        <v>0.4375</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="C14" s="2">
+        <v>12.955</v>
+      </c>
+      <c r="D14" s="2">
+        <v>77.62</v>
+      </c>
+      <c r="E14" s="2">
+        <v>12.9716</v>
+      </c>
+      <c r="F14" s="2">
+        <v>77.5946</v>
+      </c>
+      <c r="G14" s="3">
         <v>0.3333333333333333</v>
       </c>
-      <c r="H11" s="3">
-        <v>0.3611111111111111</v>
-      </c>
-      <c r="I11" s="2" t="s">
+      <c r="H14" s="3">
+        <v>0.3680555555555556</v>
+      </c>
+      <c r="I14" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="J14" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12">
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-    </row>
-    <row r="13">
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-    </row>
-    <row r="14">
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-    </row>
     <row r="15">
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
+      <c r="A15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="C15" s="2">
+        <v>12.919</v>
+      </c>
+      <c r="D15" s="2">
+        <v>77.608</v>
+      </c>
+      <c r="E15" s="2">
+        <v>12.9716</v>
+      </c>
+      <c r="F15" s="2">
+        <v>77.5946</v>
+      </c>
+      <c r="G15" s="3">
+        <v>0.40625</v>
+      </c>
+      <c r="H15" s="3">
+        <v>0.46875</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="16">
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
+      <c r="A16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="C16" s="2">
+        <v>12.948</v>
+      </c>
+      <c r="D16" s="2">
+        <v>77.635</v>
+      </c>
+      <c r="E16" s="2">
+        <v>12.9716</v>
+      </c>
+      <c r="F16" s="2">
+        <v>77.5946</v>
+      </c>
+      <c r="G16" s="3">
+        <v>0.3576388888888889</v>
+      </c>
+      <c r="H16" s="3">
+        <v>0.40625</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -876,54 +1037,54 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D2" s="2">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="E2" s="2">
         <v>10.0</v>
       </c>
       <c r="F2" s="2">
-        <v>30.0</v>
+        <v>28.0</v>
       </c>
       <c r="G2" s="2">
         <v>12.935</v>
@@ -940,22 +1101,22 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D3" s="2">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="E3" s="2">
         <v>11.0</v>
       </c>
       <c r="F3" s="2">
-        <v>28.0</v>
+        <v>30.0</v>
       </c>
       <c r="G3" s="2">
         <v>12.94</v>
@@ -972,19 +1133,19 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D4" s="2">
         <v>4.0</v>
       </c>
       <c r="E4" s="2">
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
       <c r="F4" s="2">
         <v>35.0</v>
@@ -999,24 +1160,24 @@
         <v>0.3333333333333333</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D5" s="2">
         <v>6.0</v>
       </c>
       <c r="E5" s="2">
-        <v>18.0</v>
+        <v>19.0</v>
       </c>
       <c r="F5" s="2">
         <v>32.0</v>
@@ -1031,14 +1192,72 @@
         <v>0.3333333333333333</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
-      <c r="I6" s="3"/>
+      <c r="A6" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="E6" s="2">
+        <v>8.0</v>
+      </c>
+      <c r="F6" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="G6" s="2">
+        <v>12.925</v>
+      </c>
+      <c r="H6" s="2">
+        <v>77.6</v>
+      </c>
+      <c r="I6" s="3">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
-      <c r="I7" s="3"/>
+      <c r="A7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="E7" s="2">
+        <v>14.0</v>
+      </c>
+      <c r="F7" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="G7" s="2">
+        <v>12.96</v>
+      </c>
+      <c r="H7" s="2">
+        <v>77.64</v>
+      </c>
+      <c r="I7" s="3">
+        <v>0.3402777777777778</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>18</v>
+      </c>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -1057,10 +1276,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2">
@@ -1068,10 +1287,10 @@
         <v>10</v>
       </c>
       <c r="B2" s="2">
-        <v>420.0</v>
+        <v>450.0</v>
       </c>
       <c r="C2" s="2">
-        <v>40.0</v>
+        <v>42.0</v>
       </c>
     </row>
     <row r="3">
@@ -1079,10 +1298,10 @@
         <v>13</v>
       </c>
       <c r="B3" s="2">
-        <v>425.0</v>
+        <v>440.0</v>
       </c>
       <c r="C3" s="2">
-        <v>42.0</v>
+        <v>43.0</v>
       </c>
     </row>
     <row r="4">
@@ -1090,54 +1309,54 @@
         <v>14</v>
       </c>
       <c r="B4" s="2">
-        <v>430.0</v>
+        <v>410.0</v>
       </c>
       <c r="C4" s="2">
-        <v>43.0</v>
+        <v>50.0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B5" s="2">
-        <v>435.0</v>
+        <v>390.0</v>
       </c>
       <c r="C5" s="2">
-        <v>44.0</v>
+        <v>55.0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B6" s="2">
-        <v>400.0</v>
+        <v>470.0</v>
       </c>
       <c r="C6" s="2">
-        <v>50.0</v>
+        <v>62.0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B7" s="2">
-        <v>395.0</v>
+        <v>420.0</v>
       </c>
       <c r="C7" s="2">
-        <v>50.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B8" s="2">
-        <v>380.0</v>
+        <v>460.0</v>
       </c>
       <c r="C8" s="2">
-        <v>58.0</v>
+        <v>41.0</v>
       </c>
     </row>
     <row r="9">
@@ -1145,10 +1364,10 @@
         <v>23</v>
       </c>
       <c r="B9" s="2">
-        <v>385.0</v>
+        <v>400.0</v>
       </c>
       <c r="C9" s="2">
-        <v>58.0</v>
+        <v>57.0</v>
       </c>
     </row>
     <row r="10">
@@ -1156,7 +1375,7 @@
         <v>24</v>
       </c>
       <c r="B10" s="2">
-        <v>450.0</v>
+        <v>380.0</v>
       </c>
       <c r="C10" s="2">
         <v>65.0</v>
@@ -1167,10 +1386,65 @@
         <v>25</v>
       </c>
       <c r="B11" s="2">
-        <v>700.0</v>
+        <v>455.0</v>
       </c>
       <c r="C11" s="2">
-        <v>35.0</v>
+        <v>60.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="2">
+        <v>430.0</v>
+      </c>
+      <c r="C12" s="2">
+        <v>49.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="2">
+        <v>395.0</v>
+      </c>
+      <c r="C13" s="2">
+        <v>53.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="2">
+        <v>465.0</v>
+      </c>
+      <c r="C14" s="2">
+        <v>40.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="2">
+        <v>460.0</v>
+      </c>
+      <c r="C15" s="2">
+        <v>63.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="2">
+        <v>425.0</v>
+      </c>
+      <c r="C16" s="2">
+        <v>47.0</v>
       </c>
     </row>
   </sheetData>
@@ -1184,54 +1458,50 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="21.63"/>
-    <col customWidth="1" min="2" max="2" width="16.88"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="B5" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="B6" s="2">
         <v>5.0</v>
@@ -1239,31 +1509,31 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="B7" s="2">
-        <v>10.0</v>
+        <v>8.0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B8" s="2">
-        <v>15.0</v>
+        <v>12.0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="B9" s="2">
-        <v>20.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="B10" s="2">
         <v>30.0</v>
@@ -1271,26 +1541,18 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="B11" s="2">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="B12" s="2">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="B13" s="2" t="b">
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>